<commit_message>
Polish galaxy view and manage gradual orbital traffic
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/galaxy_config.xlsx
+++ b/space-battleship/config_excel/galaxy_config.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="galaxy_config" sheetId="1" r:id="R91e35412f64343c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="galaxy_config" sheetId="1" r:id="R617a01d054c2485b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -428,6 +428,48 @@
         <x:v>最大相机缩放</x:v>
       </x:c>
     </x:row>
+    <x:row r="14">
+      <x:c r="A14" t="str">
+        <x:v>transport_buildings_per_ship</x:v>
+      </x:c>
+      <x:c r="B14" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C14" t="str">
+        <x:v>float</x:v>
+      </x:c>
+      <x:c r="D14" t="str">
+        <x:v>每艇对应已建成功能建筑（座/艇）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" t="str">
+        <x:v>transport_initial_delay</x:v>
+      </x:c>
+      <x:c r="B15" t="n">
+        <x:v>1.4</x:v>
+      </x:c>
+      <x:c r="C15" t="str">
+        <x:v>float</x:v>
+      </x:c>
+      <x:c r="D15" t="str">
+        <x:v>展示艇首次启程延迟（秒）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" t="str">
+        <x:v>transport_departure_interval</x:v>
+      </x:c>
+      <x:c r="B16" t="n">
+        <x:v>0.8</x:v>
+      </x:c>
+      <x:c r="C16" t="str">
+        <x:v>float</x:v>
+      </x:c>
+      <x:c r="D16" t="str">
+        <x:v>展示艇错峰启程间隔（秒）</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Cap city framing, connect foundation pipes and fly decorative traffic above roofs
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/galaxy_config.xlsx
+++ b/space-battleship/config_excel/galaxy_config.xlsx
@@ -377,7 +377,7 @@
         <x:v>max_transport_ships</x:v>
       </x:c>
       <x:c r="B10" t="n">
-        <x:v>12</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="C10" t="str">
         <x:v>int</x:v>
@@ -405,7 +405,7 @@
         <x:v>camera_zoom_min</x:v>
       </x:c>
       <x:c r="B12" t="n">
-        <x:v>0.6</x:v>
+        <x:v>0.4</x:v>
       </x:c>
       <x:c r="C12" t="str">
         <x:v>float</x:v>
@@ -419,7 +419,7 @@
         <x:v>camera_zoom_max</x:v>
       </x:c>
       <x:c r="B13" t="n">
-        <x:v>2.8</x:v>
+        <x:v>0.6</x:v>
       </x:c>
       <x:c r="C13" t="str">
         <x:v>float</x:v>
@@ -433,7 +433,7 @@
         <x:v>transport_buildings_per_ship</x:v>
       </x:c>
       <x:c r="B14" t="n">
-        <x:v>3</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="C14" t="str">
         <x:v>float</x:v>

</xml_diff>

<commit_message>
Build shared galaxy city districts around the central headquarters
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/galaxy_config.xlsx
+++ b/space-battleship/config_excel/galaxy_config.xlsx
@@ -377,7 +377,7 @@
         <x:v>max_transport_ships</x:v>
       </x:c>
       <x:c r="B10" t="n">
-        <x:v>12</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="C10" t="str">
         <x:v>int</x:v>
@@ -405,7 +405,7 @@
         <x:v>camera_zoom_min</x:v>
       </x:c>
       <x:c r="B12" t="n">
-        <x:v>0.6</x:v>
+        <x:v>0.4</x:v>
       </x:c>
       <x:c r="C12" t="str">
         <x:v>float</x:v>
@@ -419,7 +419,7 @@
         <x:v>camera_zoom_max</x:v>
       </x:c>
       <x:c r="B13" t="n">
-        <x:v>2.8</x:v>
+        <x:v>0.6</x:v>
       </x:c>
       <x:c r="C13" t="str">
         <x:v>float</x:v>
@@ -433,7 +433,7 @@
         <x:v>transport_buildings_per_ship</x:v>
       </x:c>
       <x:c r="B14" t="n">
-        <x:v>3</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="C14" t="str">
         <x:v>float</x:v>

</xml_diff>

<commit_message>
Integrate approved individual galaxy platforms with live building interactions
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/galaxy_config.xlsx
+++ b/space-battleship/config_excel/galaxy_config.xlsx
@@ -377,7 +377,7 @@
         <x:v>max_transport_ships</x:v>
       </x:c>
       <x:c r="B10" t="n">
-        <x:v>12</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="C10" t="str">
         <x:v>int</x:v>
@@ -405,7 +405,7 @@
         <x:v>camera_zoom_min</x:v>
       </x:c>
       <x:c r="B12" t="n">
-        <x:v>0.6</x:v>
+        <x:v>0.4</x:v>
       </x:c>
       <x:c r="C12" t="str">
         <x:v>float</x:v>
@@ -419,7 +419,7 @@
         <x:v>camera_zoom_max</x:v>
       </x:c>
       <x:c r="B13" t="n">
-        <x:v>2.8</x:v>
+        <x:v>0.6</x:v>
       </x:c>
       <x:c r="C13" t="str">
         <x:v>float</x:v>
@@ -433,7 +433,7 @@
         <x:v>transport_buildings_per_ship</x:v>
       </x:c>
       <x:c r="B14" t="n">
-        <x:v>3</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="C14" t="str">
         <x:v>float</x:v>

</xml_diff>